<commit_message>
Lady Madrid: ampliar Control de Inventario con bebidas y consumibles
El archivo solo cubría comida/obrador. Se añade BEBIDAS_OTRAS siguiendo
el mismo circuito Ventas del mes → Escandallos → Inventario (consumo
directo, cantidad 1 por unidad vendida), y un bloque nuevo CONSUMIBLES
en Inventario con seguimiento por compras y recuento (no vinculado a
ventas, ya que no se venden como plato). Escandallos_LadyMadrid.xlsx no
tiene datos reales de bebidas sin café ni de consumibles, así que las
líneas añadidas son ejemplos marcados explícitamente como tales, a la
espera del listado real de Lady Madrid.
</commit_message>
<xml_diff>
--- a/clientes/lady-madrid/run/Control_Inventario_Lady_Madrid.xlsx
+++ b/clientes/lady-madrid/run/Control_Inventario_Lady_Madrid.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -659,7 +659,7 @@
     <row r="16" ht="62" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>323 líneas de ingrediente, una por cada producto de Escandallos_LadyMadrid.xlsx. No tocar salvo que cambie una receta o se dé de alta un plato nuevo — en ese caso, añadirlo aquí Y en 'Ventas del mes' con el mismo nombre y categoría exactos.</t>
+          <t>323 líneas de ingrediente, una por cada producto de Escandallos_LadyMadrid.xlsx. No tocar salvo que cambie una receta o se dé de alta un plato nuevo — en ese caso, añadirlo aquí Y en 'Ventas del mes' con el mismo nombre y categoría exactos. (más 7 líneas de BEBIDAS_OTRAS añadidas el 2026-10-20, ver nota al final de esta pestaña).</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
     <row r="19" ht="62" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Una fila por ingrediente (168 ingredientes únicos). Rellenar solo las 3 columnas amarillas: inventario del mes anterior, compras del mes, e inventario real del mes actual (el recuento físico). Todo lo demás —consumo teórico, variación, alerta— se calcula solo.</t>
+          <t>Una fila por ingrediente (168 ingredientes únicos). Rellenar solo las 3 columnas amarillas: inventario del mes anterior, compras del mes, e inventario real del mes actual (el recuento físico). Todo lo demás —consumo teórico, variación, alerta— se calcula solo. (más 7 bebidas y el bloque de CONSUMIBLES al final de la pestaña, añadidos el 2026-10-20).</t>
         </is>
       </c>
     </row>
@@ -716,6 +716,27 @@
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>(1) 2 líneas del archivo original no eran ingredientes reales (una nota de preparación y una etiqueta de sección) — excluidas, no aparecen en 'Escandallos'. (2) 'AOVE' en CAKE CHOCOLATE, AOVE Y SAL no tiene cantidad especificada en el archivo original — queda en 0, hay que confirmarla con cocina/obrador. (3) Unidad inconsistente entre platos para 7 ingredientes (AOVE, Escamas de sal, Huevo pochado, Almendra laminada, Almendra tostada, Brioche — marcados con comentario en la pestaña Inventario). (4) Nombres casi idénticos pero no exactos entre platos (ej. 'PISTO Y YEMA CURADA' en desayunos y en tardes; variantes marcadas '(no)' que parecen descatalogadas) — no se han fusionado ni eliminado por mi cuenta, alguien de cocina tiene que confirmarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Actualización 2026-10-20 — Bebidas y consumibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Se ha ampliado esta plantilla para cubrir no solo comida/obrador sino también bebidas (más allá del café, que ya estaba cubierto en BEBIDAS_CAFÉ) y consumibles. La categoría BEBIDAS_OTRAS sigue el mismo circuito que el resto (Ventas del mes → Escandallos → Inventario): cada bebida se trata como un ingrediente de cantidad 1 por unidad vendida (consumo directo, sin receta). Los consumibles (limpieza, papel, envases) no se venden como plato, así que no pasan por 'Ventas del mes': tienen su propio bloque al final de la pestaña 'Inventario', con seguimiento directo por compras y recuento físico, sin consumo teórico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Las líneas de BEBIDAS_OTRAS y del bloque CONSUMIBLES son EJEMPLOS de referencia (formato de hostelería estándar), no el listado real de Lady Madrid — hay que sustituirlas por la carta real de bebidas y el listado real de consumibles del local antes de usar esta plantilla en producción. Pendiente: pedir a Andrea/cocina el listado real.</t>
         </is>
       </c>
     </row>
@@ -730,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1759,6 +1780,146 @@
         <v>0</v>
       </c>
       <c r="D65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>AGUA CON GAS</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>AGUA SIN GAS</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA ZERO</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>ZUMO DE NARANJA NATURAL</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>CERVEZA BOTELLÍN</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>COPA DE VINO</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por la carta real de bebidas de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1774,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G324"/>
+  <dimension ref="A1:G331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1855,7 +2016,7 @@
         </is>
       </c>
       <c r="F4" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A4)*('Ventas del mes'!$B$4:$B$65=B4)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A4)*('Ventas del mes'!$B$4:$B$72=B4)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -1888,7 +2049,7 @@
         </is>
       </c>
       <c r="F5" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A5)*('Ventas del mes'!$B$4:$B$65=B5)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A5)*('Ventas del mes'!$B$4:$B$72=B5)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G5" s="9">
@@ -1921,7 +2082,7 @@
         </is>
       </c>
       <c r="F6" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A6)*('Ventas del mes'!$B$4:$B$65=B6)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A6)*('Ventas del mes'!$B$4:$B$72=B6)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -1954,7 +2115,7 @@
         </is>
       </c>
       <c r="F7" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A7)*('Ventas del mes'!$B$4:$B$65=B7)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A7)*('Ventas del mes'!$B$4:$B$72=B7)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G7" s="9">
@@ -1987,7 +2148,7 @@
         </is>
       </c>
       <c r="F8" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A8)*('Ventas del mes'!$B$4:$B$65=B8)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A8)*('Ventas del mes'!$B$4:$B$72=B8)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -2020,7 +2181,7 @@
         </is>
       </c>
       <c r="F9" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A9)*('Ventas del mes'!$B$4:$B$65=B9)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A9)*('Ventas del mes'!$B$4:$B$72=B9)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G9" s="9">
@@ -2053,7 +2214,7 @@
         </is>
       </c>
       <c r="F10" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A10)*('Ventas del mes'!$B$4:$B$65=B10)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A10)*('Ventas del mes'!$B$4:$B$72=B10)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -2086,7 +2247,7 @@
         </is>
       </c>
       <c r="F11" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A11)*('Ventas del mes'!$B$4:$B$65=B11)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A11)*('Ventas del mes'!$B$4:$B$72=B11)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G11" s="9">
@@ -2119,7 +2280,7 @@
         </is>
       </c>
       <c r="F12" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A12)*('Ventas del mes'!$B$4:$B$65=B12)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A12)*('Ventas del mes'!$B$4:$B$72=B12)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -2152,7 +2313,7 @@
         </is>
       </c>
       <c r="F13" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A13)*('Ventas del mes'!$B$4:$B$65=B13)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A13)*('Ventas del mes'!$B$4:$B$72=B13)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G13" s="9">
@@ -2185,7 +2346,7 @@
         </is>
       </c>
       <c r="F14" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A14)*('Ventas del mes'!$B$4:$B$65=B14)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A14)*('Ventas del mes'!$B$4:$B$72=B14)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -2218,7 +2379,7 @@
         </is>
       </c>
       <c r="F15" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A15)*('Ventas del mes'!$B$4:$B$65=B15)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A15)*('Ventas del mes'!$B$4:$B$72=B15)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G15" s="9">
@@ -2251,7 +2412,7 @@
         </is>
       </c>
       <c r="F16" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A16)*('Ventas del mes'!$B$4:$B$65=B16)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A16)*('Ventas del mes'!$B$4:$B$72=B16)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -2284,7 +2445,7 @@
         </is>
       </c>
       <c r="F17" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A17)*('Ventas del mes'!$B$4:$B$65=B17)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A17)*('Ventas del mes'!$B$4:$B$72=B17)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G17" s="9">
@@ -2317,7 +2478,7 @@
         </is>
       </c>
       <c r="F18" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A18)*('Ventas del mes'!$B$4:$B$65=B18)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A18)*('Ventas del mes'!$B$4:$B$72=B18)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -2350,7 +2511,7 @@
         </is>
       </c>
       <c r="F19" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A19)*('Ventas del mes'!$B$4:$B$65=B19)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A19)*('Ventas del mes'!$B$4:$B$72=B19)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G19" s="9">
@@ -2383,7 +2544,7 @@
         </is>
       </c>
       <c r="F20" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A20)*('Ventas del mes'!$B$4:$B$65=B20)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A20)*('Ventas del mes'!$B$4:$B$72=B20)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -2416,7 +2577,7 @@
         </is>
       </c>
       <c r="F21" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A21)*('Ventas del mes'!$B$4:$B$65=B21)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A21)*('Ventas del mes'!$B$4:$B$72=B21)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G21" s="9">
@@ -2449,7 +2610,7 @@
         </is>
       </c>
       <c r="F22" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A22)*('Ventas del mes'!$B$4:$B$65=B22)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A22)*('Ventas del mes'!$B$4:$B$72=B22)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G22" s="9">
@@ -2482,7 +2643,7 @@
         </is>
       </c>
       <c r="F23" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A23)*('Ventas del mes'!$B$4:$B$65=B23)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A23)*('Ventas del mes'!$B$4:$B$72=B23)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G23" s="9">
@@ -2515,7 +2676,7 @@
         </is>
       </c>
       <c r="F24" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A24)*('Ventas del mes'!$B$4:$B$65=B24)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A24)*('Ventas del mes'!$B$4:$B$72=B24)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G24" s="9">
@@ -2548,7 +2709,7 @@
         </is>
       </c>
       <c r="F25" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A25)*('Ventas del mes'!$B$4:$B$65=B25)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A25)*('Ventas del mes'!$B$4:$B$72=B25)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G25" s="9">
@@ -2581,7 +2742,7 @@
         </is>
       </c>
       <c r="F26" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A26)*('Ventas del mes'!$B$4:$B$65=B26)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A26)*('Ventas del mes'!$B$4:$B$72=B26)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G26" s="9">
@@ -2614,7 +2775,7 @@
         </is>
       </c>
       <c r="F27" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A27)*('Ventas del mes'!$B$4:$B$65=B27)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A27)*('Ventas del mes'!$B$4:$B$72=B27)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G27" s="9">
@@ -2647,7 +2808,7 @@
         </is>
       </c>
       <c r="F28" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A28)*('Ventas del mes'!$B$4:$B$65=B28)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A28)*('Ventas del mes'!$B$4:$B$72=B28)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G28" s="9">
@@ -2680,7 +2841,7 @@
         </is>
       </c>
       <c r="F29" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A29)*('Ventas del mes'!$B$4:$B$65=B29)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A29)*('Ventas del mes'!$B$4:$B$72=B29)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G29" s="9">
@@ -2713,7 +2874,7 @@
         </is>
       </c>
       <c r="F30" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A30)*('Ventas del mes'!$B$4:$B$65=B30)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A30)*('Ventas del mes'!$B$4:$B$72=B30)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G30" s="9">
@@ -2746,7 +2907,7 @@
         </is>
       </c>
       <c r="F31" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A31)*('Ventas del mes'!$B$4:$B$65=B31)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A31)*('Ventas del mes'!$B$4:$B$72=B31)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G31" s="9">
@@ -2779,7 +2940,7 @@
         </is>
       </c>
       <c r="F32" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A32)*('Ventas del mes'!$B$4:$B$65=B32)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A32)*('Ventas del mes'!$B$4:$B$72=B32)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G32" s="9">
@@ -2812,7 +2973,7 @@
         </is>
       </c>
       <c r="F33" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A33)*('Ventas del mes'!$B$4:$B$65=B33)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A33)*('Ventas del mes'!$B$4:$B$72=B33)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G33" s="9">
@@ -2845,7 +3006,7 @@
         </is>
       </c>
       <c r="F34" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A34)*('Ventas del mes'!$B$4:$B$65=B34)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A34)*('Ventas del mes'!$B$4:$B$72=B34)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G34" s="9">
@@ -2878,7 +3039,7 @@
         </is>
       </c>
       <c r="F35" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A35)*('Ventas del mes'!$B$4:$B$65=B35)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A35)*('Ventas del mes'!$B$4:$B$72=B35)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G35" s="9">
@@ -2911,7 +3072,7 @@
         </is>
       </c>
       <c r="F36" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A36)*('Ventas del mes'!$B$4:$B$65=B36)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A36)*('Ventas del mes'!$B$4:$B$72=B36)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G36" s="9">
@@ -2944,7 +3105,7 @@
         </is>
       </c>
       <c r="F37" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A37)*('Ventas del mes'!$B$4:$B$65=B37)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A37)*('Ventas del mes'!$B$4:$B$72=B37)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G37" s="9">
@@ -2977,7 +3138,7 @@
         </is>
       </c>
       <c r="F38" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A38)*('Ventas del mes'!$B$4:$B$65=B38)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A38)*('Ventas del mes'!$B$4:$B$72=B38)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G38" s="9">
@@ -3010,7 +3171,7 @@
         </is>
       </c>
       <c r="F39" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A39)*('Ventas del mes'!$B$4:$B$65=B39)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A39)*('Ventas del mes'!$B$4:$B$72=B39)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G39" s="9">
@@ -3043,7 +3204,7 @@
         </is>
       </c>
       <c r="F40" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A40)*('Ventas del mes'!$B$4:$B$65=B40)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A40)*('Ventas del mes'!$B$4:$B$72=B40)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G40" s="9">
@@ -3076,7 +3237,7 @@
         </is>
       </c>
       <c r="F41" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A41)*('Ventas del mes'!$B$4:$B$65=B41)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A41)*('Ventas del mes'!$B$4:$B$72=B41)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G41" s="9">
@@ -3109,7 +3270,7 @@
         </is>
       </c>
       <c r="F42" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A42)*('Ventas del mes'!$B$4:$B$65=B42)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A42)*('Ventas del mes'!$B$4:$B$72=B42)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G42" s="9">
@@ -3142,7 +3303,7 @@
         </is>
       </c>
       <c r="F43" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A43)*('Ventas del mes'!$B$4:$B$65=B43)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A43)*('Ventas del mes'!$B$4:$B$72=B43)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G43" s="9">
@@ -3175,7 +3336,7 @@
         </is>
       </c>
       <c r="F44" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A44)*('Ventas del mes'!$B$4:$B$65=B44)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A44)*('Ventas del mes'!$B$4:$B$72=B44)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G44" s="9">
@@ -3208,7 +3369,7 @@
         </is>
       </c>
       <c r="F45" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A45)*('Ventas del mes'!$B$4:$B$65=B45)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A45)*('Ventas del mes'!$B$4:$B$72=B45)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G45" s="9">
@@ -3241,7 +3402,7 @@
         </is>
       </c>
       <c r="F46" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A46)*('Ventas del mes'!$B$4:$B$65=B46)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A46)*('Ventas del mes'!$B$4:$B$72=B46)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G46" s="9">
@@ -3274,7 +3435,7 @@
         </is>
       </c>
       <c r="F47" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A47)*('Ventas del mes'!$B$4:$B$65=B47)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A47)*('Ventas del mes'!$B$4:$B$72=B47)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G47" s="9">
@@ -3307,7 +3468,7 @@
         </is>
       </c>
       <c r="F48" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A48)*('Ventas del mes'!$B$4:$B$65=B48)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A48)*('Ventas del mes'!$B$4:$B$72=B48)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G48" s="9">
@@ -3340,7 +3501,7 @@
         </is>
       </c>
       <c r="F49" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A49)*('Ventas del mes'!$B$4:$B$65=B49)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A49)*('Ventas del mes'!$B$4:$B$72=B49)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G49" s="9">
@@ -3373,7 +3534,7 @@
         </is>
       </c>
       <c r="F50" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A50)*('Ventas del mes'!$B$4:$B$65=B50)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A50)*('Ventas del mes'!$B$4:$B$72=B50)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G50" s="9">
@@ -3406,7 +3567,7 @@
         </is>
       </c>
       <c r="F51" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A51)*('Ventas del mes'!$B$4:$B$65=B51)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A51)*('Ventas del mes'!$B$4:$B$72=B51)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G51" s="9">
@@ -3439,7 +3600,7 @@
         </is>
       </c>
       <c r="F52" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A52)*('Ventas del mes'!$B$4:$B$65=B52)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A52)*('Ventas del mes'!$B$4:$B$72=B52)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G52" s="9">
@@ -3472,7 +3633,7 @@
         </is>
       </c>
       <c r="F53" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A53)*('Ventas del mes'!$B$4:$B$65=B53)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A53)*('Ventas del mes'!$B$4:$B$72=B53)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G53" s="9">
@@ -3505,7 +3666,7 @@
         </is>
       </c>
       <c r="F54" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A54)*('Ventas del mes'!$B$4:$B$65=B54)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A54)*('Ventas del mes'!$B$4:$B$72=B54)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G54" s="9">
@@ -3538,7 +3699,7 @@
         </is>
       </c>
       <c r="F55" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A55)*('Ventas del mes'!$B$4:$B$65=B55)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A55)*('Ventas del mes'!$B$4:$B$72=B55)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G55" s="9">
@@ -3571,7 +3732,7 @@
         </is>
       </c>
       <c r="F56" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A56)*('Ventas del mes'!$B$4:$B$65=B56)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A56)*('Ventas del mes'!$B$4:$B$72=B56)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G56" s="9">
@@ -3604,7 +3765,7 @@
         </is>
       </c>
       <c r="F57" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A57)*('Ventas del mes'!$B$4:$B$65=B57)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A57)*('Ventas del mes'!$B$4:$B$72=B57)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G57" s="9">
@@ -3637,7 +3798,7 @@
         </is>
       </c>
       <c r="F58" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A58)*('Ventas del mes'!$B$4:$B$65=B58)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A58)*('Ventas del mes'!$B$4:$B$72=B58)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G58" s="9">
@@ -3670,7 +3831,7 @@
         </is>
       </c>
       <c r="F59" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A59)*('Ventas del mes'!$B$4:$B$65=B59)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A59)*('Ventas del mes'!$B$4:$B$72=B59)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G59" s="9">
@@ -3703,7 +3864,7 @@
         </is>
       </c>
       <c r="F60" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A60)*('Ventas del mes'!$B$4:$B$65=B60)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A60)*('Ventas del mes'!$B$4:$B$72=B60)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G60" s="9">
@@ -3736,7 +3897,7 @@
         </is>
       </c>
       <c r="F61" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A61)*('Ventas del mes'!$B$4:$B$65=B61)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A61)*('Ventas del mes'!$B$4:$B$72=B61)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G61" s="9">
@@ -3769,7 +3930,7 @@
         </is>
       </c>
       <c r="F62" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A62)*('Ventas del mes'!$B$4:$B$65=B62)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A62)*('Ventas del mes'!$B$4:$B$72=B62)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G62" s="9">
@@ -3802,7 +3963,7 @@
         </is>
       </c>
       <c r="F63" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A63)*('Ventas del mes'!$B$4:$B$65=B63)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A63)*('Ventas del mes'!$B$4:$B$72=B63)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G63" s="9">
@@ -3835,7 +3996,7 @@
         </is>
       </c>
       <c r="F64" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A64)*('Ventas del mes'!$B$4:$B$65=B64)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A64)*('Ventas del mes'!$B$4:$B$72=B64)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G64" s="9">
@@ -3868,7 +4029,7 @@
         </is>
       </c>
       <c r="F65" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A65)*('Ventas del mes'!$B$4:$B$65=B65)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A65)*('Ventas del mes'!$B$4:$B$72=B65)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G65" s="9">
@@ -3901,7 +4062,7 @@
         </is>
       </c>
       <c r="F66" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A66)*('Ventas del mes'!$B$4:$B$65=B66)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A66)*('Ventas del mes'!$B$4:$B$72=B66)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G66" s="9">
@@ -3934,7 +4095,7 @@
         </is>
       </c>
       <c r="F67" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A67)*('Ventas del mes'!$B$4:$B$65=B67)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A67)*('Ventas del mes'!$B$4:$B$72=B67)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G67" s="9">
@@ -3967,7 +4128,7 @@
         </is>
       </c>
       <c r="F68" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A68)*('Ventas del mes'!$B$4:$B$65=B68)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A68)*('Ventas del mes'!$B$4:$B$72=B68)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G68" s="9">
@@ -4000,7 +4161,7 @@
         </is>
       </c>
       <c r="F69" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A69)*('Ventas del mes'!$B$4:$B$65=B69)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A69)*('Ventas del mes'!$B$4:$B$72=B69)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G69" s="9">
@@ -4033,7 +4194,7 @@
         </is>
       </c>
       <c r="F70" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A70)*('Ventas del mes'!$B$4:$B$65=B70)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A70)*('Ventas del mes'!$B$4:$B$72=B70)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G70" s="9">
@@ -4066,7 +4227,7 @@
         </is>
       </c>
       <c r="F71" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A71)*('Ventas del mes'!$B$4:$B$65=B71)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A71)*('Ventas del mes'!$B$4:$B$72=B71)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G71" s="9">
@@ -4099,7 +4260,7 @@
         </is>
       </c>
       <c r="F72" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A72)*('Ventas del mes'!$B$4:$B$65=B72)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A72)*('Ventas del mes'!$B$4:$B$72=B72)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G72" s="9">
@@ -4132,7 +4293,7 @@
         </is>
       </c>
       <c r="F73" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A73)*('Ventas del mes'!$B$4:$B$65=B73)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A73)*('Ventas del mes'!$B$4:$B$72=B73)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G73" s="9">
@@ -4165,7 +4326,7 @@
         </is>
       </c>
       <c r="F74" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A74)*('Ventas del mes'!$B$4:$B$65=B74)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A74)*('Ventas del mes'!$B$4:$B$72=B74)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G74" s="9">
@@ -4198,7 +4359,7 @@
         </is>
       </c>
       <c r="F75" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A75)*('Ventas del mes'!$B$4:$B$65=B75)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A75)*('Ventas del mes'!$B$4:$B$72=B75)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G75" s="9">
@@ -4231,7 +4392,7 @@
         </is>
       </c>
       <c r="F76" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A76)*('Ventas del mes'!$B$4:$B$65=B76)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A76)*('Ventas del mes'!$B$4:$B$72=B76)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G76" s="9">
@@ -4264,7 +4425,7 @@
         </is>
       </c>
       <c r="F77" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A77)*('Ventas del mes'!$B$4:$B$65=B77)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A77)*('Ventas del mes'!$B$4:$B$72=B77)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G77" s="9">
@@ -4297,7 +4458,7 @@
         </is>
       </c>
       <c r="F78" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A78)*('Ventas del mes'!$B$4:$B$65=B78)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A78)*('Ventas del mes'!$B$4:$B$72=B78)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G78" s="9">
@@ -4330,7 +4491,7 @@
         </is>
       </c>
       <c r="F79" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A79)*('Ventas del mes'!$B$4:$B$65=B79)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A79)*('Ventas del mes'!$B$4:$B$72=B79)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G79" s="9">
@@ -4363,7 +4524,7 @@
         </is>
       </c>
       <c r="F80" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A80)*('Ventas del mes'!$B$4:$B$65=B80)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A80)*('Ventas del mes'!$B$4:$B$72=B80)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G80" s="9">
@@ -4396,7 +4557,7 @@
         </is>
       </c>
       <c r="F81" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A81)*('Ventas del mes'!$B$4:$B$65=B81)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A81)*('Ventas del mes'!$B$4:$B$72=B81)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G81" s="9">
@@ -4429,7 +4590,7 @@
         </is>
       </c>
       <c r="F82" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A82)*('Ventas del mes'!$B$4:$B$65=B82)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A82)*('Ventas del mes'!$B$4:$B$72=B82)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G82" s="9">
@@ -4462,7 +4623,7 @@
         </is>
       </c>
       <c r="F83" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A83)*('Ventas del mes'!$B$4:$B$65=B83)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A83)*('Ventas del mes'!$B$4:$B$72=B83)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G83" s="9">
@@ -4495,7 +4656,7 @@
         </is>
       </c>
       <c r="F84" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A84)*('Ventas del mes'!$B$4:$B$65=B84)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A84)*('Ventas del mes'!$B$4:$B$72=B84)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G84" s="9">
@@ -4528,7 +4689,7 @@
         </is>
       </c>
       <c r="F85" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A85)*('Ventas del mes'!$B$4:$B$65=B85)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A85)*('Ventas del mes'!$B$4:$B$72=B85)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G85" s="9">
@@ -4561,7 +4722,7 @@
         </is>
       </c>
       <c r="F86" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A86)*('Ventas del mes'!$B$4:$B$65=B86)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A86)*('Ventas del mes'!$B$4:$B$72=B86)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G86" s="9">
@@ -4594,7 +4755,7 @@
         </is>
       </c>
       <c r="F87" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A87)*('Ventas del mes'!$B$4:$B$65=B87)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A87)*('Ventas del mes'!$B$4:$B$72=B87)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G87" s="9">
@@ -4627,7 +4788,7 @@
         </is>
       </c>
       <c r="F88" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A88)*('Ventas del mes'!$B$4:$B$65=B88)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A88)*('Ventas del mes'!$B$4:$B$72=B88)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G88" s="9">
@@ -4660,7 +4821,7 @@
         </is>
       </c>
       <c r="F89" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A89)*('Ventas del mes'!$B$4:$B$65=B89)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A89)*('Ventas del mes'!$B$4:$B$72=B89)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
@@ -4693,7 +4854,7 @@
         </is>
       </c>
       <c r="F90" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A90)*('Ventas del mes'!$B$4:$B$65=B90)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A90)*('Ventas del mes'!$B$4:$B$72=B90)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G90" s="9">
@@ -4726,7 +4887,7 @@
         </is>
       </c>
       <c r="F91" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A91)*('Ventas del mes'!$B$4:$B$65=B91)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A91)*('Ventas del mes'!$B$4:$B$72=B91)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G91" s="9">
@@ -4759,7 +4920,7 @@
         </is>
       </c>
       <c r="F92" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A92)*('Ventas del mes'!$B$4:$B$65=B92)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A92)*('Ventas del mes'!$B$4:$B$72=B92)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G92" s="9">
@@ -4792,7 +4953,7 @@
         </is>
       </c>
       <c r="F93" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A93)*('Ventas del mes'!$B$4:$B$65=B93)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A93)*('Ventas del mes'!$B$4:$B$72=B93)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G93" s="9">
@@ -4825,7 +4986,7 @@
         </is>
       </c>
       <c r="F94" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A94)*('Ventas del mes'!$B$4:$B$65=B94)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A94)*('Ventas del mes'!$B$4:$B$72=B94)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G94" s="9">
@@ -4858,7 +5019,7 @@
         </is>
       </c>
       <c r="F95" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A95)*('Ventas del mes'!$B$4:$B$65=B95)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A95)*('Ventas del mes'!$B$4:$B$72=B95)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G95" s="9">
@@ -4891,7 +5052,7 @@
         </is>
       </c>
       <c r="F96" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A96)*('Ventas del mes'!$B$4:$B$65=B96)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A96)*('Ventas del mes'!$B$4:$B$72=B96)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G96" s="9">
@@ -4924,7 +5085,7 @@
         </is>
       </c>
       <c r="F97" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A97)*('Ventas del mes'!$B$4:$B$65=B97)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A97)*('Ventas del mes'!$B$4:$B$72=B97)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G97" s="9">
@@ -4957,7 +5118,7 @@
         </is>
       </c>
       <c r="F98" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A98)*('Ventas del mes'!$B$4:$B$65=B98)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A98)*('Ventas del mes'!$B$4:$B$72=B98)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
@@ -4990,7 +5151,7 @@
         </is>
       </c>
       <c r="F99" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A99)*('Ventas del mes'!$B$4:$B$65=B99)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A99)*('Ventas del mes'!$B$4:$B$72=B99)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G99" s="9">
@@ -5023,7 +5184,7 @@
         </is>
       </c>
       <c r="F100" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A100)*('Ventas del mes'!$B$4:$B$65=B100)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A100)*('Ventas del mes'!$B$4:$B$72=B100)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G100" s="9">
@@ -5056,7 +5217,7 @@
         </is>
       </c>
       <c r="F101" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A101)*('Ventas del mes'!$B$4:$B$65=B101)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A101)*('Ventas del mes'!$B$4:$B$72=B101)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G101" s="9">
@@ -5089,7 +5250,7 @@
         </is>
       </c>
       <c r="F102" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A102)*('Ventas del mes'!$B$4:$B$65=B102)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A102)*('Ventas del mes'!$B$4:$B$72=B102)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G102" s="9">
@@ -5122,7 +5283,7 @@
         </is>
       </c>
       <c r="F103" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A103)*('Ventas del mes'!$B$4:$B$65=B103)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A103)*('Ventas del mes'!$B$4:$B$72=B103)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G103" s="9">
@@ -5155,7 +5316,7 @@
         </is>
       </c>
       <c r="F104" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A104)*('Ventas del mes'!$B$4:$B$65=B104)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A104)*('Ventas del mes'!$B$4:$B$72=B104)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G104" s="9">
@@ -5188,7 +5349,7 @@
         </is>
       </c>
       <c r="F105" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A105)*('Ventas del mes'!$B$4:$B$65=B105)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A105)*('Ventas del mes'!$B$4:$B$72=B105)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G105" s="9">
@@ -5221,7 +5382,7 @@
         </is>
       </c>
       <c r="F106" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A106)*('Ventas del mes'!$B$4:$B$65=B106)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A106)*('Ventas del mes'!$B$4:$B$72=B106)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G106" s="9">
@@ -5254,7 +5415,7 @@
         </is>
       </c>
       <c r="F107" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A107)*('Ventas del mes'!$B$4:$B$65=B107)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A107)*('Ventas del mes'!$B$4:$B$72=B107)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G107" s="9">
@@ -5287,7 +5448,7 @@
         </is>
       </c>
       <c r="F108" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A108)*('Ventas del mes'!$B$4:$B$65=B108)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A108)*('Ventas del mes'!$B$4:$B$72=B108)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G108" s="9">
@@ -5320,7 +5481,7 @@
         </is>
       </c>
       <c r="F109" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A109)*('Ventas del mes'!$B$4:$B$65=B109)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A109)*('Ventas del mes'!$B$4:$B$72=B109)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G109" s="9">
@@ -5353,7 +5514,7 @@
         </is>
       </c>
       <c r="F110" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A110)*('Ventas del mes'!$B$4:$B$65=B110)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A110)*('Ventas del mes'!$B$4:$B$72=B110)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G110" s="9">
@@ -5386,7 +5547,7 @@
         </is>
       </c>
       <c r="F111" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A111)*('Ventas del mes'!$B$4:$B$65=B111)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A111)*('Ventas del mes'!$B$4:$B$72=B111)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G111" s="9">
@@ -5419,7 +5580,7 @@
         </is>
       </c>
       <c r="F112" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A112)*('Ventas del mes'!$B$4:$B$65=B112)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A112)*('Ventas del mes'!$B$4:$B$72=B112)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G112" s="9">
@@ -5452,7 +5613,7 @@
         </is>
       </c>
       <c r="F113" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A113)*('Ventas del mes'!$B$4:$B$65=B113)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A113)*('Ventas del mes'!$B$4:$B$72=B113)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G113" s="9">
@@ -5485,7 +5646,7 @@
         </is>
       </c>
       <c r="F114" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A114)*('Ventas del mes'!$B$4:$B$65=B114)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A114)*('Ventas del mes'!$B$4:$B$72=B114)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G114" s="9">
@@ -5518,7 +5679,7 @@
         </is>
       </c>
       <c r="F115" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A115)*('Ventas del mes'!$B$4:$B$65=B115)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A115)*('Ventas del mes'!$B$4:$B$72=B115)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G115" s="9">
@@ -5551,7 +5712,7 @@
         </is>
       </c>
       <c r="F116" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A116)*('Ventas del mes'!$B$4:$B$65=B116)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A116)*('Ventas del mes'!$B$4:$B$72=B116)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G116" s="9">
@@ -5584,7 +5745,7 @@
         </is>
       </c>
       <c r="F117" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A117)*('Ventas del mes'!$B$4:$B$65=B117)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A117)*('Ventas del mes'!$B$4:$B$72=B117)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G117" s="9">
@@ -5617,7 +5778,7 @@
         </is>
       </c>
       <c r="F118" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A118)*('Ventas del mes'!$B$4:$B$65=B118)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A118)*('Ventas del mes'!$B$4:$B$72=B118)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G118" s="9">
@@ -5650,7 +5811,7 @@
         </is>
       </c>
       <c r="F119" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A119)*('Ventas del mes'!$B$4:$B$65=B119)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A119)*('Ventas del mes'!$B$4:$B$72=B119)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G119" s="9">
@@ -5683,7 +5844,7 @@
         </is>
       </c>
       <c r="F120" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A120)*('Ventas del mes'!$B$4:$B$65=B120)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A120)*('Ventas del mes'!$B$4:$B$72=B120)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G120" s="9">
@@ -5716,7 +5877,7 @@
         </is>
       </c>
       <c r="F121" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A121)*('Ventas del mes'!$B$4:$B$65=B121)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A121)*('Ventas del mes'!$B$4:$B$72=B121)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G121" s="9">
@@ -5749,7 +5910,7 @@
         </is>
       </c>
       <c r="F122" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A122)*('Ventas del mes'!$B$4:$B$65=B122)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A122)*('Ventas del mes'!$B$4:$B$72=B122)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G122" s="9">
@@ -5782,7 +5943,7 @@
         </is>
       </c>
       <c r="F123" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A123)*('Ventas del mes'!$B$4:$B$65=B123)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A123)*('Ventas del mes'!$B$4:$B$72=B123)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G123" s="9">
@@ -5815,7 +5976,7 @@
         </is>
       </c>
       <c r="F124" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A124)*('Ventas del mes'!$B$4:$B$65=B124)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A124)*('Ventas del mes'!$B$4:$B$72=B124)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G124" s="9">
@@ -5848,7 +6009,7 @@
         </is>
       </c>
       <c r="F125" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A125)*('Ventas del mes'!$B$4:$B$65=B125)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A125)*('Ventas del mes'!$B$4:$B$72=B125)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G125" s="9">
@@ -5881,7 +6042,7 @@
         </is>
       </c>
       <c r="F126" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A126)*('Ventas del mes'!$B$4:$B$65=B126)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A126)*('Ventas del mes'!$B$4:$B$72=B126)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G126" s="9">
@@ -5914,7 +6075,7 @@
         </is>
       </c>
       <c r="F127" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A127)*('Ventas del mes'!$B$4:$B$65=B127)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A127)*('Ventas del mes'!$B$4:$B$72=B127)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G127" s="9">
@@ -5947,7 +6108,7 @@
         </is>
       </c>
       <c r="F128" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A128)*('Ventas del mes'!$B$4:$B$65=B128)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A128)*('Ventas del mes'!$B$4:$B$72=B128)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G128" s="9">
@@ -5980,7 +6141,7 @@
         </is>
       </c>
       <c r="F129" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A129)*('Ventas del mes'!$B$4:$B$65=B129)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A129)*('Ventas del mes'!$B$4:$B$72=B129)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G129" s="9">
@@ -6013,7 +6174,7 @@
         </is>
       </c>
       <c r="F130" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A130)*('Ventas del mes'!$B$4:$B$65=B130)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A130)*('Ventas del mes'!$B$4:$B$72=B130)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G130" s="9">
@@ -6046,7 +6207,7 @@
         </is>
       </c>
       <c r="F131" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A131)*('Ventas del mes'!$B$4:$B$65=B131)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A131)*('Ventas del mes'!$B$4:$B$72=B131)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G131" s="9">
@@ -6079,7 +6240,7 @@
         </is>
       </c>
       <c r="F132" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A132)*('Ventas del mes'!$B$4:$B$65=B132)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A132)*('Ventas del mes'!$B$4:$B$72=B132)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G132" s="9">
@@ -6112,7 +6273,7 @@
         </is>
       </c>
       <c r="F133" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A133)*('Ventas del mes'!$B$4:$B$65=B133)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A133)*('Ventas del mes'!$B$4:$B$72=B133)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G133" s="9">
@@ -6145,7 +6306,7 @@
         </is>
       </c>
       <c r="F134" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A134)*('Ventas del mes'!$B$4:$B$65=B134)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A134)*('Ventas del mes'!$B$4:$B$72=B134)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G134" s="9">
@@ -6178,7 +6339,7 @@
         </is>
       </c>
       <c r="F135" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A135)*('Ventas del mes'!$B$4:$B$65=B135)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A135)*('Ventas del mes'!$B$4:$B$72=B135)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G135" s="9">
@@ -6211,7 +6372,7 @@
         </is>
       </c>
       <c r="F136" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A136)*('Ventas del mes'!$B$4:$B$65=B136)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A136)*('Ventas del mes'!$B$4:$B$72=B136)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G136" s="9">
@@ -6244,7 +6405,7 @@
         </is>
       </c>
       <c r="F137" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A137)*('Ventas del mes'!$B$4:$B$65=B137)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A137)*('Ventas del mes'!$B$4:$B$72=B137)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G137" s="9">
@@ -6277,7 +6438,7 @@
         </is>
       </c>
       <c r="F138" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A138)*('Ventas del mes'!$B$4:$B$65=B138)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A138)*('Ventas del mes'!$B$4:$B$72=B138)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G138" s="9">
@@ -6310,7 +6471,7 @@
         </is>
       </c>
       <c r="F139" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A139)*('Ventas del mes'!$B$4:$B$65=B139)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A139)*('Ventas del mes'!$B$4:$B$72=B139)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G139" s="9">
@@ -6343,7 +6504,7 @@
         </is>
       </c>
       <c r="F140" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A140)*('Ventas del mes'!$B$4:$B$65=B140)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A140)*('Ventas del mes'!$B$4:$B$72=B140)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G140" s="9">
@@ -6376,7 +6537,7 @@
         </is>
       </c>
       <c r="F141" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A141)*('Ventas del mes'!$B$4:$B$65=B141)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A141)*('Ventas del mes'!$B$4:$B$72=B141)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G141" s="9">
@@ -6409,7 +6570,7 @@
         </is>
       </c>
       <c r="F142" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A142)*('Ventas del mes'!$B$4:$B$65=B142)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A142)*('Ventas del mes'!$B$4:$B$72=B142)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G142" s="9">
@@ -6442,7 +6603,7 @@
         </is>
       </c>
       <c r="F143" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A143)*('Ventas del mes'!$B$4:$B$65=B143)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A143)*('Ventas del mes'!$B$4:$B$72=B143)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G143" s="9">
@@ -6475,7 +6636,7 @@
         </is>
       </c>
       <c r="F144" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A144)*('Ventas del mes'!$B$4:$B$65=B144)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A144)*('Ventas del mes'!$B$4:$B$72=B144)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G144" s="9">
@@ -6508,7 +6669,7 @@
         </is>
       </c>
       <c r="F145" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A145)*('Ventas del mes'!$B$4:$B$65=B145)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A145)*('Ventas del mes'!$B$4:$B$72=B145)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G145" s="9">
@@ -6541,7 +6702,7 @@
         </is>
       </c>
       <c r="F146" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A146)*('Ventas del mes'!$B$4:$B$65=B146)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A146)*('Ventas del mes'!$B$4:$B$72=B146)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G146" s="9">
@@ -6574,7 +6735,7 @@
         </is>
       </c>
       <c r="F147" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A147)*('Ventas del mes'!$B$4:$B$65=B147)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A147)*('Ventas del mes'!$B$4:$B$72=B147)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G147" s="9">
@@ -6607,7 +6768,7 @@
         </is>
       </c>
       <c r="F148" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A148)*('Ventas del mes'!$B$4:$B$65=B148)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A148)*('Ventas del mes'!$B$4:$B$72=B148)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G148" s="9">
@@ -6640,7 +6801,7 @@
         </is>
       </c>
       <c r="F149" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A149)*('Ventas del mes'!$B$4:$B$65=B149)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A149)*('Ventas del mes'!$B$4:$B$72=B149)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G149" s="9">
@@ -6673,7 +6834,7 @@
         </is>
       </c>
       <c r="F150" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A150)*('Ventas del mes'!$B$4:$B$65=B150)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A150)*('Ventas del mes'!$B$4:$B$72=B150)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G150" s="9">
@@ -6706,7 +6867,7 @@
         </is>
       </c>
       <c r="F151" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A151)*('Ventas del mes'!$B$4:$B$65=B151)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A151)*('Ventas del mes'!$B$4:$B$72=B151)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G151" s="9">
@@ -6739,7 +6900,7 @@
         </is>
       </c>
       <c r="F152" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A152)*('Ventas del mes'!$B$4:$B$65=B152)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A152)*('Ventas del mes'!$B$4:$B$72=B152)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G152" s="9">
@@ -6772,7 +6933,7 @@
         </is>
       </c>
       <c r="F153" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A153)*('Ventas del mes'!$B$4:$B$65=B153)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A153)*('Ventas del mes'!$B$4:$B$72=B153)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G153" s="9">
@@ -6805,7 +6966,7 @@
         </is>
       </c>
       <c r="F154" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A154)*('Ventas del mes'!$B$4:$B$65=B154)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A154)*('Ventas del mes'!$B$4:$B$72=B154)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G154" s="9">
@@ -6838,7 +6999,7 @@
         </is>
       </c>
       <c r="F155" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A155)*('Ventas del mes'!$B$4:$B$65=B155)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A155)*('Ventas del mes'!$B$4:$B$72=B155)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G155" s="9">
@@ -6871,7 +7032,7 @@
         </is>
       </c>
       <c r="F156" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A156)*('Ventas del mes'!$B$4:$B$65=B156)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A156)*('Ventas del mes'!$B$4:$B$72=B156)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G156" s="9">
@@ -6904,7 +7065,7 @@
         </is>
       </c>
       <c r="F157" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A157)*('Ventas del mes'!$B$4:$B$65=B157)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A157)*('Ventas del mes'!$B$4:$B$72=B157)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G157" s="9">
@@ -6937,7 +7098,7 @@
         </is>
       </c>
       <c r="F158" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A158)*('Ventas del mes'!$B$4:$B$65=B158)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A158)*('Ventas del mes'!$B$4:$B$72=B158)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G158" s="9">
@@ -6970,7 +7131,7 @@
         </is>
       </c>
       <c r="F159" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A159)*('Ventas del mes'!$B$4:$B$65=B159)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A159)*('Ventas del mes'!$B$4:$B$72=B159)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G159" s="9">
@@ -7003,7 +7164,7 @@
         </is>
       </c>
       <c r="F160" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A160)*('Ventas del mes'!$B$4:$B$65=B160)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A160)*('Ventas del mes'!$B$4:$B$72=B160)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G160" s="9">
@@ -7036,7 +7197,7 @@
         </is>
       </c>
       <c r="F161" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A161)*('Ventas del mes'!$B$4:$B$65=B161)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A161)*('Ventas del mes'!$B$4:$B$72=B161)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G161" s="9">
@@ -7069,7 +7230,7 @@
         </is>
       </c>
       <c r="F162" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A162)*('Ventas del mes'!$B$4:$B$65=B162)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A162)*('Ventas del mes'!$B$4:$B$72=B162)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G162" s="9">
@@ -7102,7 +7263,7 @@
         </is>
       </c>
       <c r="F163" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A163)*('Ventas del mes'!$B$4:$B$65=B163)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A163)*('Ventas del mes'!$B$4:$B$72=B163)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G163" s="9">
@@ -7135,7 +7296,7 @@
         </is>
       </c>
       <c r="F164" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A164)*('Ventas del mes'!$B$4:$B$65=B164)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A164)*('Ventas del mes'!$B$4:$B$72=B164)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G164" s="9">
@@ -7168,7 +7329,7 @@
         </is>
       </c>
       <c r="F165" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A165)*('Ventas del mes'!$B$4:$B$65=B165)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A165)*('Ventas del mes'!$B$4:$B$72=B165)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G165" s="9">
@@ -7201,7 +7362,7 @@
         </is>
       </c>
       <c r="F166" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A166)*('Ventas del mes'!$B$4:$B$65=B166)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A166)*('Ventas del mes'!$B$4:$B$72=B166)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G166" s="9">
@@ -7234,7 +7395,7 @@
         </is>
       </c>
       <c r="F167" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A167)*('Ventas del mes'!$B$4:$B$65=B167)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A167)*('Ventas del mes'!$B$4:$B$72=B167)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G167" s="9">
@@ -7267,7 +7428,7 @@
         </is>
       </c>
       <c r="F168" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A168)*('Ventas del mes'!$B$4:$B$65=B168)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A168)*('Ventas del mes'!$B$4:$B$72=B168)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G168" s="9">
@@ -7300,7 +7461,7 @@
         </is>
       </c>
       <c r="F169" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A169)*('Ventas del mes'!$B$4:$B$65=B169)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A169)*('Ventas del mes'!$B$4:$B$72=B169)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G169" s="9">
@@ -7333,7 +7494,7 @@
         </is>
       </c>
       <c r="F170" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A170)*('Ventas del mes'!$B$4:$B$65=B170)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A170)*('Ventas del mes'!$B$4:$B$72=B170)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G170" s="9">
@@ -7366,7 +7527,7 @@
         </is>
       </c>
       <c r="F171" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A171)*('Ventas del mes'!$B$4:$B$65=B171)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A171)*('Ventas del mes'!$B$4:$B$72=B171)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G171" s="9">
@@ -7399,7 +7560,7 @@
         </is>
       </c>
       <c r="F172" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A172)*('Ventas del mes'!$B$4:$B$65=B172)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A172)*('Ventas del mes'!$B$4:$B$72=B172)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G172" s="9">
@@ -7432,7 +7593,7 @@
         </is>
       </c>
       <c r="F173" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A173)*('Ventas del mes'!$B$4:$B$65=B173)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A173)*('Ventas del mes'!$B$4:$B$72=B173)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G173" s="9">
@@ -7465,7 +7626,7 @@
         </is>
       </c>
       <c r="F174" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A174)*('Ventas del mes'!$B$4:$B$65=B174)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A174)*('Ventas del mes'!$B$4:$B$72=B174)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G174" s="9">
@@ -7498,7 +7659,7 @@
         </is>
       </c>
       <c r="F175" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A175)*('Ventas del mes'!$B$4:$B$65=B175)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A175)*('Ventas del mes'!$B$4:$B$72=B175)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G175" s="9">
@@ -7531,7 +7692,7 @@
         </is>
       </c>
       <c r="F176" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A176)*('Ventas del mes'!$B$4:$B$65=B176)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A176)*('Ventas del mes'!$B$4:$B$72=B176)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G176" s="9">
@@ -7564,7 +7725,7 @@
         </is>
       </c>
       <c r="F177" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A177)*('Ventas del mes'!$B$4:$B$65=B177)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A177)*('Ventas del mes'!$B$4:$B$72=B177)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G177" s="9">
@@ -7597,7 +7758,7 @@
         </is>
       </c>
       <c r="F178" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A178)*('Ventas del mes'!$B$4:$B$65=B178)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A178)*('Ventas del mes'!$B$4:$B$72=B178)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G178" s="9">
@@ -7630,7 +7791,7 @@
         </is>
       </c>
       <c r="F179" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A179)*('Ventas del mes'!$B$4:$B$65=B179)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A179)*('Ventas del mes'!$B$4:$B$72=B179)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G179" s="9">
@@ -7663,7 +7824,7 @@
         </is>
       </c>
       <c r="F180" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A180)*('Ventas del mes'!$B$4:$B$65=B180)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A180)*('Ventas del mes'!$B$4:$B$72=B180)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G180" s="9">
@@ -7696,7 +7857,7 @@
         </is>
       </c>
       <c r="F181" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A181)*('Ventas del mes'!$B$4:$B$65=B181)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A181)*('Ventas del mes'!$B$4:$B$72=B181)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G181" s="9">
@@ -7729,7 +7890,7 @@
         </is>
       </c>
       <c r="F182" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A182)*('Ventas del mes'!$B$4:$B$65=B182)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A182)*('Ventas del mes'!$B$4:$B$72=B182)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G182" s="9">
@@ -7762,7 +7923,7 @@
         </is>
       </c>
       <c r="F183" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A183)*('Ventas del mes'!$B$4:$B$65=B183)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A183)*('Ventas del mes'!$B$4:$B$72=B183)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G183" s="9">
@@ -7795,7 +7956,7 @@
         </is>
       </c>
       <c r="F184" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A184)*('Ventas del mes'!$B$4:$B$65=B184)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A184)*('Ventas del mes'!$B$4:$B$72=B184)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G184" s="9">
@@ -7828,7 +7989,7 @@
         </is>
       </c>
       <c r="F185" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A185)*('Ventas del mes'!$B$4:$B$65=B185)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A185)*('Ventas del mes'!$B$4:$B$72=B185)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G185" s="9">
@@ -7861,7 +8022,7 @@
         </is>
       </c>
       <c r="F186" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A186)*('Ventas del mes'!$B$4:$B$65=B186)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A186)*('Ventas del mes'!$B$4:$B$72=B186)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G186" s="9">
@@ -7894,7 +8055,7 @@
         </is>
       </c>
       <c r="F187" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A187)*('Ventas del mes'!$B$4:$B$65=B187)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A187)*('Ventas del mes'!$B$4:$B$72=B187)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G187" s="9">
@@ -7927,7 +8088,7 @@
         </is>
       </c>
       <c r="F188" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A188)*('Ventas del mes'!$B$4:$B$65=B188)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A188)*('Ventas del mes'!$B$4:$B$72=B188)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G188" s="9">
@@ -7960,7 +8121,7 @@
         </is>
       </c>
       <c r="F189" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A189)*('Ventas del mes'!$B$4:$B$65=B189)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A189)*('Ventas del mes'!$B$4:$B$72=B189)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G189" s="9">
@@ -7993,7 +8154,7 @@
         </is>
       </c>
       <c r="F190" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A190)*('Ventas del mes'!$B$4:$B$65=B190)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A190)*('Ventas del mes'!$B$4:$B$72=B190)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G190" s="9">
@@ -8026,7 +8187,7 @@
         </is>
       </c>
       <c r="F191" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A191)*('Ventas del mes'!$B$4:$B$65=B191)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A191)*('Ventas del mes'!$B$4:$B$72=B191)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G191" s="9">
@@ -8059,7 +8220,7 @@
         </is>
       </c>
       <c r="F192" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A192)*('Ventas del mes'!$B$4:$B$65=B192)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A192)*('Ventas del mes'!$B$4:$B$72=B192)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G192" s="9">
@@ -8092,7 +8253,7 @@
         </is>
       </c>
       <c r="F193" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A193)*('Ventas del mes'!$B$4:$B$65=B193)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A193)*('Ventas del mes'!$B$4:$B$72=B193)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G193" s="9">
@@ -8125,7 +8286,7 @@
         </is>
       </c>
       <c r="F194" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A194)*('Ventas del mes'!$B$4:$B$65=B194)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A194)*('Ventas del mes'!$B$4:$B$72=B194)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G194" s="9">
@@ -8158,7 +8319,7 @@
         </is>
       </c>
       <c r="F195" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A195)*('Ventas del mes'!$B$4:$B$65=B195)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A195)*('Ventas del mes'!$B$4:$B$72=B195)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G195" s="9">
@@ -8191,7 +8352,7 @@
         </is>
       </c>
       <c r="F196" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A196)*('Ventas del mes'!$B$4:$B$65=B196)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A196)*('Ventas del mes'!$B$4:$B$72=B196)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G196" s="9">
@@ -8224,7 +8385,7 @@
         </is>
       </c>
       <c r="F197" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A197)*('Ventas del mes'!$B$4:$B$65=B197)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A197)*('Ventas del mes'!$B$4:$B$72=B197)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G197" s="9">
@@ -8257,7 +8418,7 @@
         </is>
       </c>
       <c r="F198" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A198)*('Ventas del mes'!$B$4:$B$65=B198)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A198)*('Ventas del mes'!$B$4:$B$72=B198)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G198" s="9">
@@ -8290,7 +8451,7 @@
         </is>
       </c>
       <c r="F199" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A199)*('Ventas del mes'!$B$4:$B$65=B199)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A199)*('Ventas del mes'!$B$4:$B$72=B199)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G199" s="9">
@@ -8323,7 +8484,7 @@
         </is>
       </c>
       <c r="F200" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A200)*('Ventas del mes'!$B$4:$B$65=B200)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A200)*('Ventas del mes'!$B$4:$B$72=B200)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G200" s="9">
@@ -8356,7 +8517,7 @@
         </is>
       </c>
       <c r="F201" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A201)*('Ventas del mes'!$B$4:$B$65=B201)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A201)*('Ventas del mes'!$B$4:$B$72=B201)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G201" s="9">
@@ -8389,7 +8550,7 @@
         </is>
       </c>
       <c r="F202" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A202)*('Ventas del mes'!$B$4:$B$65=B202)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A202)*('Ventas del mes'!$B$4:$B$72=B202)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G202" s="9">
@@ -8422,7 +8583,7 @@
         </is>
       </c>
       <c r="F203" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A203)*('Ventas del mes'!$B$4:$B$65=B203)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A203)*('Ventas del mes'!$B$4:$B$72=B203)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G203" s="9">
@@ -8455,7 +8616,7 @@
         </is>
       </c>
       <c r="F204" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A204)*('Ventas del mes'!$B$4:$B$65=B204)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A204)*('Ventas del mes'!$B$4:$B$72=B204)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G204" s="9">
@@ -8488,7 +8649,7 @@
         </is>
       </c>
       <c r="F205" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A205)*('Ventas del mes'!$B$4:$B$65=B205)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A205)*('Ventas del mes'!$B$4:$B$72=B205)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G205" s="9">
@@ -8521,7 +8682,7 @@
         </is>
       </c>
       <c r="F206" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A206)*('Ventas del mes'!$B$4:$B$65=B206)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A206)*('Ventas del mes'!$B$4:$B$72=B206)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G206" s="9">
@@ -8554,7 +8715,7 @@
         </is>
       </c>
       <c r="F207" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A207)*('Ventas del mes'!$B$4:$B$65=B207)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A207)*('Ventas del mes'!$B$4:$B$72=B207)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G207" s="9">
@@ -8587,7 +8748,7 @@
         </is>
       </c>
       <c r="F208" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A208)*('Ventas del mes'!$B$4:$B$65=B208)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A208)*('Ventas del mes'!$B$4:$B$72=B208)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G208" s="9">
@@ -8620,7 +8781,7 @@
         </is>
       </c>
       <c r="F209" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A209)*('Ventas del mes'!$B$4:$B$65=B209)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A209)*('Ventas del mes'!$B$4:$B$72=B209)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G209" s="9">
@@ -8653,7 +8814,7 @@
         </is>
       </c>
       <c r="F210" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A210)*('Ventas del mes'!$B$4:$B$65=B210)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A210)*('Ventas del mes'!$B$4:$B$72=B210)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G210" s="9">
@@ -8686,7 +8847,7 @@
         </is>
       </c>
       <c r="F211" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A211)*('Ventas del mes'!$B$4:$B$65=B211)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A211)*('Ventas del mes'!$B$4:$B$72=B211)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G211" s="9">
@@ -8719,7 +8880,7 @@
         </is>
       </c>
       <c r="F212" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A212)*('Ventas del mes'!$B$4:$B$65=B212)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A212)*('Ventas del mes'!$B$4:$B$72=B212)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G212" s="9">
@@ -8752,7 +8913,7 @@
         </is>
       </c>
       <c r="F213" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A213)*('Ventas del mes'!$B$4:$B$65=B213)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A213)*('Ventas del mes'!$B$4:$B$72=B213)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G213" s="9">
@@ -8785,7 +8946,7 @@
         </is>
       </c>
       <c r="F214" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A214)*('Ventas del mes'!$B$4:$B$65=B214)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A214)*('Ventas del mes'!$B$4:$B$72=B214)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G214" s="9">
@@ -8818,7 +8979,7 @@
         </is>
       </c>
       <c r="F215" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A215)*('Ventas del mes'!$B$4:$B$65=B215)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A215)*('Ventas del mes'!$B$4:$B$72=B215)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G215" s="9">
@@ -8851,7 +9012,7 @@
         </is>
       </c>
       <c r="F216" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A216)*('Ventas del mes'!$B$4:$B$65=B216)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A216)*('Ventas del mes'!$B$4:$B$72=B216)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G216" s="9">
@@ -8884,7 +9045,7 @@
         </is>
       </c>
       <c r="F217" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A217)*('Ventas del mes'!$B$4:$B$65=B217)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A217)*('Ventas del mes'!$B$4:$B$72=B217)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G217" s="9">
@@ -8917,7 +9078,7 @@
         </is>
       </c>
       <c r="F218" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A218)*('Ventas del mes'!$B$4:$B$65=B218)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A218)*('Ventas del mes'!$B$4:$B$72=B218)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G218" s="9">
@@ -8950,7 +9111,7 @@
         </is>
       </c>
       <c r="F219" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A219)*('Ventas del mes'!$B$4:$B$65=B219)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A219)*('Ventas del mes'!$B$4:$B$72=B219)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G219" s="9">
@@ -8983,7 +9144,7 @@
         </is>
       </c>
       <c r="F220" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A220)*('Ventas del mes'!$B$4:$B$65=B220)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A220)*('Ventas del mes'!$B$4:$B$72=B220)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G220" s="9">
@@ -9016,7 +9177,7 @@
         </is>
       </c>
       <c r="F221" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A221)*('Ventas del mes'!$B$4:$B$65=B221)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A221)*('Ventas del mes'!$B$4:$B$72=B221)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G221" s="9">
@@ -9049,7 +9210,7 @@
         </is>
       </c>
       <c r="F222" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A222)*('Ventas del mes'!$B$4:$B$65=B222)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A222)*('Ventas del mes'!$B$4:$B$72=B222)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G222" s="9">
@@ -9082,7 +9243,7 @@
         </is>
       </c>
       <c r="F223" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A223)*('Ventas del mes'!$B$4:$B$65=B223)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A223)*('Ventas del mes'!$B$4:$B$72=B223)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G223" s="9">
@@ -9115,7 +9276,7 @@
         </is>
       </c>
       <c r="F224" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A224)*('Ventas del mes'!$B$4:$B$65=B224)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A224)*('Ventas del mes'!$B$4:$B$72=B224)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G224" s="9">
@@ -9148,7 +9309,7 @@
         </is>
       </c>
       <c r="F225" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A225)*('Ventas del mes'!$B$4:$B$65=B225)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A225)*('Ventas del mes'!$B$4:$B$72=B225)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G225" s="9">
@@ -9181,7 +9342,7 @@
         </is>
       </c>
       <c r="F226" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A226)*('Ventas del mes'!$B$4:$B$65=B226)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A226)*('Ventas del mes'!$B$4:$B$72=B226)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G226" s="9">
@@ -9214,7 +9375,7 @@
         </is>
       </c>
       <c r="F227" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A227)*('Ventas del mes'!$B$4:$B$65=B227)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A227)*('Ventas del mes'!$B$4:$B$72=B227)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G227" s="9">
@@ -9247,7 +9408,7 @@
         </is>
       </c>
       <c r="F228" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A228)*('Ventas del mes'!$B$4:$B$65=B228)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A228)*('Ventas del mes'!$B$4:$B$72=B228)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G228" s="9">
@@ -9280,7 +9441,7 @@
         </is>
       </c>
       <c r="F229" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A229)*('Ventas del mes'!$B$4:$B$65=B229)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A229)*('Ventas del mes'!$B$4:$B$72=B229)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G229" s="9">
@@ -9313,7 +9474,7 @@
         </is>
       </c>
       <c r="F230" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A230)*('Ventas del mes'!$B$4:$B$65=B230)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A230)*('Ventas del mes'!$B$4:$B$72=B230)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G230" s="9">
@@ -9346,7 +9507,7 @@
         </is>
       </c>
       <c r="F231" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A231)*('Ventas del mes'!$B$4:$B$65=B231)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A231)*('Ventas del mes'!$B$4:$B$72=B231)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G231" s="9">
@@ -9379,7 +9540,7 @@
         </is>
       </c>
       <c r="F232" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A232)*('Ventas del mes'!$B$4:$B$65=B232)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A232)*('Ventas del mes'!$B$4:$B$72=B232)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G232" s="9">
@@ -9412,7 +9573,7 @@
         </is>
       </c>
       <c r="F233" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A233)*('Ventas del mes'!$B$4:$B$65=B233)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A233)*('Ventas del mes'!$B$4:$B$72=B233)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G233" s="9">
@@ -9445,7 +9606,7 @@
         </is>
       </c>
       <c r="F234" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A234)*('Ventas del mes'!$B$4:$B$65=B234)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A234)*('Ventas del mes'!$B$4:$B$72=B234)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G234" s="9">
@@ -9478,7 +9639,7 @@
         </is>
       </c>
       <c r="F235" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A235)*('Ventas del mes'!$B$4:$B$65=B235)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A235)*('Ventas del mes'!$B$4:$B$72=B235)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G235" s="9">
@@ -9511,7 +9672,7 @@
         </is>
       </c>
       <c r="F236" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A236)*('Ventas del mes'!$B$4:$B$65=B236)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A236)*('Ventas del mes'!$B$4:$B$72=B236)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G236" s="9">
@@ -9544,7 +9705,7 @@
         </is>
       </c>
       <c r="F237" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A237)*('Ventas del mes'!$B$4:$B$65=B237)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A237)*('Ventas del mes'!$B$4:$B$72=B237)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G237" s="9">
@@ -9577,7 +9738,7 @@
         </is>
       </c>
       <c r="F238" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A238)*('Ventas del mes'!$B$4:$B$65=B238)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A238)*('Ventas del mes'!$B$4:$B$72=B238)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G238" s="9">
@@ -9610,7 +9771,7 @@
         </is>
       </c>
       <c r="F239" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A239)*('Ventas del mes'!$B$4:$B$65=B239)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A239)*('Ventas del mes'!$B$4:$B$72=B239)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G239" s="9">
@@ -9643,7 +9804,7 @@
         </is>
       </c>
       <c r="F240" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A240)*('Ventas del mes'!$B$4:$B$65=B240)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A240)*('Ventas del mes'!$B$4:$B$72=B240)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G240" s="9">
@@ -9676,7 +9837,7 @@
         </is>
       </c>
       <c r="F241" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A241)*('Ventas del mes'!$B$4:$B$65=B241)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A241)*('Ventas del mes'!$B$4:$B$72=B241)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G241" s="9">
@@ -9709,7 +9870,7 @@
         </is>
       </c>
       <c r="F242" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A242)*('Ventas del mes'!$B$4:$B$65=B242)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A242)*('Ventas del mes'!$B$4:$B$72=B242)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G242" s="9">
@@ -9742,7 +9903,7 @@
         </is>
       </c>
       <c r="F243" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A243)*('Ventas del mes'!$B$4:$B$65=B243)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A243)*('Ventas del mes'!$B$4:$B$72=B243)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G243" s="9">
@@ -9775,7 +9936,7 @@
         </is>
       </c>
       <c r="F244" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A244)*('Ventas del mes'!$B$4:$B$65=B244)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A244)*('Ventas del mes'!$B$4:$B$72=B244)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G244" s="9">
@@ -9808,7 +9969,7 @@
         </is>
       </c>
       <c r="F245" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A245)*('Ventas del mes'!$B$4:$B$65=B245)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A245)*('Ventas del mes'!$B$4:$B$72=B245)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G245" s="9">
@@ -9841,7 +10002,7 @@
         </is>
       </c>
       <c r="F246" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A246)*('Ventas del mes'!$B$4:$B$65=B246)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A246)*('Ventas del mes'!$B$4:$B$72=B246)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G246" s="9">
@@ -9874,7 +10035,7 @@
         </is>
       </c>
       <c r="F247" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A247)*('Ventas del mes'!$B$4:$B$65=B247)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A247)*('Ventas del mes'!$B$4:$B$72=B247)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G247" s="9">
@@ -9907,7 +10068,7 @@
         </is>
       </c>
       <c r="F248" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A248)*('Ventas del mes'!$B$4:$B$65=B248)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A248)*('Ventas del mes'!$B$4:$B$72=B248)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G248" s="9">
@@ -9940,7 +10101,7 @@
         </is>
       </c>
       <c r="F249" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A249)*('Ventas del mes'!$B$4:$B$65=B249)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A249)*('Ventas del mes'!$B$4:$B$72=B249)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G249" s="9">
@@ -9973,7 +10134,7 @@
         </is>
       </c>
       <c r="F250" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A250)*('Ventas del mes'!$B$4:$B$65=B250)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A250)*('Ventas del mes'!$B$4:$B$72=B250)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G250" s="9">
@@ -10006,7 +10167,7 @@
         </is>
       </c>
       <c r="F251" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A251)*('Ventas del mes'!$B$4:$B$65=B251)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A251)*('Ventas del mes'!$B$4:$B$72=B251)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G251" s="9">
@@ -10039,7 +10200,7 @@
         </is>
       </c>
       <c r="F252" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A252)*('Ventas del mes'!$B$4:$B$65=B252)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A252)*('Ventas del mes'!$B$4:$B$72=B252)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G252" s="9">
@@ -10072,7 +10233,7 @@
         </is>
       </c>
       <c r="F253" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A253)*('Ventas del mes'!$B$4:$B$65=B253)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A253)*('Ventas del mes'!$B$4:$B$72=B253)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G253" s="9">
@@ -10105,7 +10266,7 @@
         </is>
       </c>
       <c r="F254" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A254)*('Ventas del mes'!$B$4:$B$65=B254)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A254)*('Ventas del mes'!$B$4:$B$72=B254)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G254" s="9">
@@ -10138,7 +10299,7 @@
         </is>
       </c>
       <c r="F255" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A255)*('Ventas del mes'!$B$4:$B$65=B255)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A255)*('Ventas del mes'!$B$4:$B$72=B255)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G255" s="9">
@@ -10171,7 +10332,7 @@
         </is>
       </c>
       <c r="F256" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A256)*('Ventas del mes'!$B$4:$B$65=B256)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A256)*('Ventas del mes'!$B$4:$B$72=B256)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G256" s="9">
@@ -10204,7 +10365,7 @@
         </is>
       </c>
       <c r="F257" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A257)*('Ventas del mes'!$B$4:$B$65=B257)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A257)*('Ventas del mes'!$B$4:$B$72=B257)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G257" s="9">
@@ -10237,7 +10398,7 @@
         </is>
       </c>
       <c r="F258" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A258)*('Ventas del mes'!$B$4:$B$65=B258)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A258)*('Ventas del mes'!$B$4:$B$72=B258)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G258" s="9">
@@ -10270,7 +10431,7 @@
         </is>
       </c>
       <c r="F259" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A259)*('Ventas del mes'!$B$4:$B$65=B259)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A259)*('Ventas del mes'!$B$4:$B$72=B259)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G259" s="9">
@@ -10303,7 +10464,7 @@
         </is>
       </c>
       <c r="F260" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A260)*('Ventas del mes'!$B$4:$B$65=B260)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A260)*('Ventas del mes'!$B$4:$B$72=B260)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G260" s="9">
@@ -10336,7 +10497,7 @@
         </is>
       </c>
       <c r="F261" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A261)*('Ventas del mes'!$B$4:$B$65=B261)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A261)*('Ventas del mes'!$B$4:$B$72=B261)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G261" s="9">
@@ -10369,7 +10530,7 @@
         </is>
       </c>
       <c r="F262" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A262)*('Ventas del mes'!$B$4:$B$65=B262)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A262)*('Ventas del mes'!$B$4:$B$72=B262)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G262" s="9">
@@ -10402,7 +10563,7 @@
         </is>
       </c>
       <c r="F263" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A263)*('Ventas del mes'!$B$4:$B$65=B263)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A263)*('Ventas del mes'!$B$4:$B$72=B263)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G263" s="9">
@@ -10435,7 +10596,7 @@
         </is>
       </c>
       <c r="F264" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A264)*('Ventas del mes'!$B$4:$B$65=B264)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A264)*('Ventas del mes'!$B$4:$B$72=B264)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G264" s="9">
@@ -10468,7 +10629,7 @@
         </is>
       </c>
       <c r="F265" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A265)*('Ventas del mes'!$B$4:$B$65=B265)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A265)*('Ventas del mes'!$B$4:$B$72=B265)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G265" s="9">
@@ -10501,7 +10662,7 @@
         </is>
       </c>
       <c r="F266" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A266)*('Ventas del mes'!$B$4:$B$65=B266)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A266)*('Ventas del mes'!$B$4:$B$72=B266)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G266" s="9">
@@ -10534,7 +10695,7 @@
         </is>
       </c>
       <c r="F267" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A267)*('Ventas del mes'!$B$4:$B$65=B267)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A267)*('Ventas del mes'!$B$4:$B$72=B267)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G267" s="9">
@@ -10567,7 +10728,7 @@
         </is>
       </c>
       <c r="F268" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A268)*('Ventas del mes'!$B$4:$B$65=B268)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A268)*('Ventas del mes'!$B$4:$B$72=B268)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G268" s="9">
@@ -10600,7 +10761,7 @@
         </is>
       </c>
       <c r="F269" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A269)*('Ventas del mes'!$B$4:$B$65=B269)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A269)*('Ventas del mes'!$B$4:$B$72=B269)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G269" s="9">
@@ -10633,7 +10794,7 @@
         </is>
       </c>
       <c r="F270" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A270)*('Ventas del mes'!$B$4:$B$65=B270)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A270)*('Ventas del mes'!$B$4:$B$72=B270)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G270" s="9">
@@ -10666,7 +10827,7 @@
         </is>
       </c>
       <c r="F271" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A271)*('Ventas del mes'!$B$4:$B$65=B271)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A271)*('Ventas del mes'!$B$4:$B$72=B271)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G271" s="9">
@@ -10699,7 +10860,7 @@
         </is>
       </c>
       <c r="F272" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A272)*('Ventas del mes'!$B$4:$B$65=B272)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A272)*('Ventas del mes'!$B$4:$B$72=B272)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G272" s="9">
@@ -10732,7 +10893,7 @@
         </is>
       </c>
       <c r="F273" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A273)*('Ventas del mes'!$B$4:$B$65=B273)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A273)*('Ventas del mes'!$B$4:$B$72=B273)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G273" s="9">
@@ -10765,7 +10926,7 @@
         </is>
       </c>
       <c r="F274" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A274)*('Ventas del mes'!$B$4:$B$65=B274)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A274)*('Ventas del mes'!$B$4:$B$72=B274)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G274" s="9">
@@ -10798,7 +10959,7 @@
         </is>
       </c>
       <c r="F275" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A275)*('Ventas del mes'!$B$4:$B$65=B275)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A275)*('Ventas del mes'!$B$4:$B$72=B275)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G275" s="9">
@@ -10831,7 +10992,7 @@
         </is>
       </c>
       <c r="F276" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A276)*('Ventas del mes'!$B$4:$B$65=B276)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A276)*('Ventas del mes'!$B$4:$B$72=B276)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G276" s="9">
@@ -10864,7 +11025,7 @@
         </is>
       </c>
       <c r="F277" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A277)*('Ventas del mes'!$B$4:$B$65=B277)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A277)*('Ventas del mes'!$B$4:$B$72=B277)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G277" s="9">
@@ -10897,7 +11058,7 @@
         </is>
       </c>
       <c r="F278" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A278)*('Ventas del mes'!$B$4:$B$65=B278)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A278)*('Ventas del mes'!$B$4:$B$72=B278)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G278" s="9">
@@ -10930,7 +11091,7 @@
         </is>
       </c>
       <c r="F279" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A279)*('Ventas del mes'!$B$4:$B$65=B279)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A279)*('Ventas del mes'!$B$4:$B$72=B279)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G279" s="9">
@@ -10963,7 +11124,7 @@
         </is>
       </c>
       <c r="F280" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A280)*('Ventas del mes'!$B$4:$B$65=B280)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A280)*('Ventas del mes'!$B$4:$B$72=B280)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G280" s="9">
@@ -10996,7 +11157,7 @@
         </is>
       </c>
       <c r="F281" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A281)*('Ventas del mes'!$B$4:$B$65=B281)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A281)*('Ventas del mes'!$B$4:$B$72=B281)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G281" s="9">
@@ -11029,7 +11190,7 @@
         </is>
       </c>
       <c r="F282" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A282)*('Ventas del mes'!$B$4:$B$65=B282)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A282)*('Ventas del mes'!$B$4:$B$72=B282)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G282" s="9">
@@ -11062,7 +11223,7 @@
         </is>
       </c>
       <c r="F283" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A283)*('Ventas del mes'!$B$4:$B$65=B283)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A283)*('Ventas del mes'!$B$4:$B$72=B283)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G283" s="9">
@@ -11095,7 +11256,7 @@
         </is>
       </c>
       <c r="F284" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A284)*('Ventas del mes'!$B$4:$B$65=B284)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A284)*('Ventas del mes'!$B$4:$B$72=B284)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G284" s="9">
@@ -11128,7 +11289,7 @@
         </is>
       </c>
       <c r="F285" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A285)*('Ventas del mes'!$B$4:$B$65=B285)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A285)*('Ventas del mes'!$B$4:$B$72=B285)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G285" s="9">
@@ -11161,7 +11322,7 @@
         </is>
       </c>
       <c r="F286" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A286)*('Ventas del mes'!$B$4:$B$65=B286)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A286)*('Ventas del mes'!$B$4:$B$72=B286)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G286" s="9">
@@ -11194,7 +11355,7 @@
         </is>
       </c>
       <c r="F287" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A287)*('Ventas del mes'!$B$4:$B$65=B287)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A287)*('Ventas del mes'!$B$4:$B$72=B287)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G287" s="9">
@@ -11227,7 +11388,7 @@
         </is>
       </c>
       <c r="F288" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A288)*('Ventas del mes'!$B$4:$B$65=B288)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A288)*('Ventas del mes'!$B$4:$B$72=B288)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G288" s="9">
@@ -11260,7 +11421,7 @@
         </is>
       </c>
       <c r="F289" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A289)*('Ventas del mes'!$B$4:$B$65=B289)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A289)*('Ventas del mes'!$B$4:$B$72=B289)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G289" s="9">
@@ -11293,7 +11454,7 @@
         </is>
       </c>
       <c r="F290" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A290)*('Ventas del mes'!$B$4:$B$65=B290)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A290)*('Ventas del mes'!$B$4:$B$72=B290)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G290" s="9">
@@ -11326,7 +11487,7 @@
         </is>
       </c>
       <c r="F291" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A291)*('Ventas del mes'!$B$4:$B$65=B291)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A291)*('Ventas del mes'!$B$4:$B$72=B291)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G291" s="9">
@@ -11359,7 +11520,7 @@
         </is>
       </c>
       <c r="F292" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A292)*('Ventas del mes'!$B$4:$B$65=B292)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A292)*('Ventas del mes'!$B$4:$B$72=B292)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G292" s="9">
@@ -11392,7 +11553,7 @@
         </is>
       </c>
       <c r="F293" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A293)*('Ventas del mes'!$B$4:$B$65=B293)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A293)*('Ventas del mes'!$B$4:$B$72=B293)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G293" s="9">
@@ -11425,7 +11586,7 @@
         </is>
       </c>
       <c r="F294" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A294)*('Ventas del mes'!$B$4:$B$65=B294)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A294)*('Ventas del mes'!$B$4:$B$72=B294)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G294" s="9">
@@ -11458,7 +11619,7 @@
         </is>
       </c>
       <c r="F295" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A295)*('Ventas del mes'!$B$4:$B$65=B295)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A295)*('Ventas del mes'!$B$4:$B$72=B295)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G295" s="9">
@@ -11491,7 +11652,7 @@
         </is>
       </c>
       <c r="F296" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A296)*('Ventas del mes'!$B$4:$B$65=B296)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A296)*('Ventas del mes'!$B$4:$B$72=B296)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G296" s="9">
@@ -11524,7 +11685,7 @@
         </is>
       </c>
       <c r="F297" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A297)*('Ventas del mes'!$B$4:$B$65=B297)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A297)*('Ventas del mes'!$B$4:$B$72=B297)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G297" s="9">
@@ -11557,7 +11718,7 @@
         </is>
       </c>
       <c r="F298" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A298)*('Ventas del mes'!$B$4:$B$65=B298)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A298)*('Ventas del mes'!$B$4:$B$72=B298)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G298" s="9">
@@ -11590,7 +11751,7 @@
         </is>
       </c>
       <c r="F299" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A299)*('Ventas del mes'!$B$4:$B$65=B299)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A299)*('Ventas del mes'!$B$4:$B$72=B299)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G299" s="9">
@@ -11623,7 +11784,7 @@
         </is>
       </c>
       <c r="F300" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A300)*('Ventas del mes'!$B$4:$B$65=B300)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A300)*('Ventas del mes'!$B$4:$B$72=B300)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G300" s="9">
@@ -11656,7 +11817,7 @@
         </is>
       </c>
       <c r="F301" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A301)*('Ventas del mes'!$B$4:$B$65=B301)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A301)*('Ventas del mes'!$B$4:$B$72=B301)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G301" s="9">
@@ -11689,7 +11850,7 @@
         </is>
       </c>
       <c r="F302" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A302)*('Ventas del mes'!$B$4:$B$65=B302)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A302)*('Ventas del mes'!$B$4:$B$72=B302)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G302" s="9">
@@ -11722,7 +11883,7 @@
         </is>
       </c>
       <c r="F303" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A303)*('Ventas del mes'!$B$4:$B$65=B303)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A303)*('Ventas del mes'!$B$4:$B$72=B303)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G303" s="9">
@@ -11755,7 +11916,7 @@
         </is>
       </c>
       <c r="F304" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A304)*('Ventas del mes'!$B$4:$B$65=B304)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A304)*('Ventas del mes'!$B$4:$B$72=B304)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G304" s="9">
@@ -11788,7 +11949,7 @@
         </is>
       </c>
       <c r="F305" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A305)*('Ventas del mes'!$B$4:$B$65=B305)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A305)*('Ventas del mes'!$B$4:$B$72=B305)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G305" s="9">
@@ -11821,7 +11982,7 @@
         </is>
       </c>
       <c r="F306" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A306)*('Ventas del mes'!$B$4:$B$65=B306)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A306)*('Ventas del mes'!$B$4:$B$72=B306)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G306" s="9">
@@ -11854,7 +12015,7 @@
         </is>
       </c>
       <c r="F307" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A307)*('Ventas del mes'!$B$4:$B$65=B307)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A307)*('Ventas del mes'!$B$4:$B$72=B307)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G307" s="9">
@@ -11887,7 +12048,7 @@
         </is>
       </c>
       <c r="F308" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A308)*('Ventas del mes'!$B$4:$B$65=B308)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A308)*('Ventas del mes'!$B$4:$B$72=B308)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G308" s="9">
@@ -11920,7 +12081,7 @@
         </is>
       </c>
       <c r="F309" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A309)*('Ventas del mes'!$B$4:$B$65=B309)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A309)*('Ventas del mes'!$B$4:$B$72=B309)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G309" s="9">
@@ -11953,7 +12114,7 @@
         </is>
       </c>
       <c r="F310" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A310)*('Ventas del mes'!$B$4:$B$65=B310)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A310)*('Ventas del mes'!$B$4:$B$72=B310)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G310" s="9">
@@ -11986,7 +12147,7 @@
         </is>
       </c>
       <c r="F311" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A311)*('Ventas del mes'!$B$4:$B$65=B311)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A311)*('Ventas del mes'!$B$4:$B$72=B311)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G311" s="9">
@@ -12019,7 +12180,7 @@
         </is>
       </c>
       <c r="F312" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A312)*('Ventas del mes'!$B$4:$B$65=B312)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A312)*('Ventas del mes'!$B$4:$B$72=B312)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G312" s="9">
@@ -12052,7 +12213,7 @@
         </is>
       </c>
       <c r="F313" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A313)*('Ventas del mes'!$B$4:$B$65=B313)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A313)*('Ventas del mes'!$B$4:$B$72=B313)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G313" s="9">
@@ -12085,7 +12246,7 @@
         </is>
       </c>
       <c r="F314" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A314)*('Ventas del mes'!$B$4:$B$65=B314)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A314)*('Ventas del mes'!$B$4:$B$72=B314)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G314" s="9">
@@ -12118,7 +12279,7 @@
         </is>
       </c>
       <c r="F315" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A315)*('Ventas del mes'!$B$4:$B$65=B315)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A315)*('Ventas del mes'!$B$4:$B$72=B315)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G315" s="9">
@@ -12151,7 +12312,7 @@
         </is>
       </c>
       <c r="F316" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A316)*('Ventas del mes'!$B$4:$B$65=B316)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A316)*('Ventas del mes'!$B$4:$B$72=B316)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G316" s="9">
@@ -12184,7 +12345,7 @@
         </is>
       </c>
       <c r="F317" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A317)*('Ventas del mes'!$B$4:$B$65=B317)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A317)*('Ventas del mes'!$B$4:$B$72=B317)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G317" s="9">
@@ -12217,7 +12378,7 @@
         </is>
       </c>
       <c r="F318" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A318)*('Ventas del mes'!$B$4:$B$65=B318)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A318)*('Ventas del mes'!$B$4:$B$72=B318)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G318" s="9">
@@ -12250,7 +12411,7 @@
         </is>
       </c>
       <c r="F319" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A319)*('Ventas del mes'!$B$4:$B$65=B319)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A319)*('Ventas del mes'!$B$4:$B$72=B319)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G319" s="9">
@@ -12283,7 +12444,7 @@
         </is>
       </c>
       <c r="F320" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A320)*('Ventas del mes'!$B$4:$B$65=B320)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A320)*('Ventas del mes'!$B$4:$B$72=B320)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G320" s="9">
@@ -12316,7 +12477,7 @@
         </is>
       </c>
       <c r="F321" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A321)*('Ventas del mes'!$B$4:$B$65=B321)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A321)*('Ventas del mes'!$B$4:$B$72=B321)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G321" s="9">
@@ -12349,7 +12510,7 @@
         </is>
       </c>
       <c r="F322" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A322)*('Ventas del mes'!$B$4:$B$65=B322)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A322)*('Ventas del mes'!$B$4:$B$72=B322)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G322" s="9">
@@ -12382,7 +12543,7 @@
         </is>
       </c>
       <c r="F323" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A323)*('Ventas del mes'!$B$4:$B$65=B323)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A323)*('Ventas del mes'!$B$4:$B$72=B323)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G323" s="9">
@@ -12415,11 +12576,242 @@
         </is>
       </c>
       <c r="F324" s="6">
-        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$65=A324)*('Ventas del mes'!$B$4:$B$65=B324)*'Ventas del mes'!$C$4:$C$65),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A324)*('Ventas del mes'!$B$4:$B$72=B324)*'Ventas del mes'!$C$4:$C$72),0)</f>
         <v/>
       </c>
       <c r="G324" s="9">
         <f>D324*F324</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B325" s="6" t="inlineStr">
+        <is>
+          <t>AGUA CON GAS</t>
+        </is>
+      </c>
+      <c r="C325" s="6" t="inlineStr">
+        <is>
+          <t>AGUA CON GAS</t>
+        </is>
+      </c>
+      <c r="D325" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E325" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F325" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A325)*('Ventas del mes'!$B$4:$B$72=B325)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G325" s="9">
+        <f>D325*F325</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B326" s="6" t="inlineStr">
+        <is>
+          <t>AGUA SIN GAS</t>
+        </is>
+      </c>
+      <c r="C326" s="6" t="inlineStr">
+        <is>
+          <t>AGUA SIN GAS</t>
+        </is>
+      </c>
+      <c r="D326" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E326" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F326" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A326)*('Ventas del mes'!$B$4:$B$72=B326)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G326" s="9">
+        <f>D326*F326</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B327" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA</t>
+        </is>
+      </c>
+      <c r="C327" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA</t>
+        </is>
+      </c>
+      <c r="D327" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E327" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F327" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A327)*('Ventas del mes'!$B$4:$B$72=B327)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G327" s="9">
+        <f>D327*F327</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B328" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA ZERO</t>
+        </is>
+      </c>
+      <c r="C328" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA ZERO</t>
+        </is>
+      </c>
+      <c r="D328" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E328" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F328" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A328)*('Ventas del mes'!$B$4:$B$72=B328)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G328" s="9">
+        <f>D328*F328</f>
+        <v/>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B329" s="6" t="inlineStr">
+        <is>
+          <t>ZUMO DE NARANJA NATURAL</t>
+        </is>
+      </c>
+      <c r="C329" s="6" t="inlineStr">
+        <is>
+          <t>ZUMO DE NARANJA NATURAL</t>
+        </is>
+      </c>
+      <c r="D329" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E329" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F329" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A329)*('Ventas del mes'!$B$4:$B$72=B329)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G329" s="9">
+        <f>D329*F329</f>
+        <v/>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B330" s="6" t="inlineStr">
+        <is>
+          <t>CERVEZA BOTELLÍN</t>
+        </is>
+      </c>
+      <c r="C330" s="6" t="inlineStr">
+        <is>
+          <t>CERVEZA BOTELLÍN</t>
+        </is>
+      </c>
+      <c r="D330" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E330" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F330" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A330)*('Ventas del mes'!$B$4:$B$72=B330)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G330" s="9">
+        <f>D330*F330</f>
+        <v/>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="6" t="inlineStr">
+        <is>
+          <t>BEBIDAS_OTRAS</t>
+        </is>
+      </c>
+      <c r="B331" s="6" t="inlineStr">
+        <is>
+          <t>COPA DE VINO</t>
+        </is>
+      </c>
+      <c r="C331" s="6" t="inlineStr">
+        <is>
+          <t>COPA DE VINO</t>
+        </is>
+      </c>
+      <c r="D331" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E331" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="F331" s="6">
+        <f>IFERROR(SUMPRODUCT(('Ventas del mes'!$A$4:$A$72=A331)*('Ventas del mes'!$B$4:$B$72=B331)*'Ventas del mes'!$C$4:$C$72),0)</f>
+        <v/>
+      </c>
+      <c r="G331" s="9">
+        <f>D331*F331</f>
         <v/>
       </c>
     </row>
@@ -12438,7 +12830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J172"/>
+  <dimension ref="A1:J190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -19328,44 +19720,615 @@
         <v/>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>AGUA CON GAS</t>
+        </is>
+      </c>
+      <c r="B171" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A171,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F171" s="9">
+        <f>C171+D171-E171</f>
+        <v/>
+      </c>
+      <c r="G171" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" s="9">
+        <f>G171-F171</f>
+        <v/>
+      </c>
+      <c r="I171" s="14">
+        <f>IFERROR(H171/F171,0)</f>
+        <v/>
+      </c>
+      <c r="J171" s="15">
+        <f>IF(ABS(I171)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
     <row r="172">
-      <c r="A172" s="11" t="inlineStr">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>AGUA SIN GAS</t>
+        </is>
+      </c>
+      <c r="B172" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E172" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A172,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F172" s="9">
+        <f>C172+D172-E172</f>
+        <v/>
+      </c>
+      <c r="G172" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" s="9">
+        <f>G172-F172</f>
+        <v/>
+      </c>
+      <c r="I172" s="14">
+        <f>IFERROR(H172/F172,0)</f>
+        <v/>
+      </c>
+      <c r="J172" s="15">
+        <f>IF(ABS(I172)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA</t>
+        </is>
+      </c>
+      <c r="B173" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C173" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A173,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F173" s="9">
+        <f>C173+D173-E173</f>
+        <v/>
+      </c>
+      <c r="G173" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" s="9">
+        <f>G173-F173</f>
+        <v/>
+      </c>
+      <c r="I173" s="14">
+        <f>IFERROR(H173/F173,0)</f>
+        <v/>
+      </c>
+      <c r="J173" s="15">
+        <f>IF(ABS(I173)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>REFRESCO DE COLA ZERO</t>
+        </is>
+      </c>
+      <c r="B174" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A174,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F174" s="9">
+        <f>C174+D174-E174</f>
+        <v/>
+      </c>
+      <c r="G174" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" s="9">
+        <f>G174-F174</f>
+        <v/>
+      </c>
+      <c r="I174" s="14">
+        <f>IFERROR(H174/F174,0)</f>
+        <v/>
+      </c>
+      <c r="J174" s="15">
+        <f>IF(ABS(I174)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>ZUMO DE NARANJA NATURAL</t>
+        </is>
+      </c>
+      <c r="B175" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D175" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A175,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F175" s="9">
+        <f>C175+D175-E175</f>
+        <v/>
+      </c>
+      <c r="G175" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" s="9">
+        <f>G175-F175</f>
+        <v/>
+      </c>
+      <c r="I175" s="14">
+        <f>IFERROR(H175/F175,0)</f>
+        <v/>
+      </c>
+      <c r="J175" s="15">
+        <f>IF(ABS(I175)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>CERVEZA BOTELLÍN</t>
+        </is>
+      </c>
+      <c r="B176" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A176,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F176" s="9">
+        <f>C176+D176-E176</f>
+        <v/>
+      </c>
+      <c r="G176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="9">
+        <f>G176-F176</f>
+        <v/>
+      </c>
+      <c r="I176" s="14">
+        <f>IFERROR(H176/F176,0)</f>
+        <v/>
+      </c>
+      <c r="J176" s="15">
+        <f>IF(ABS(I176)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>COPA DE VINO</t>
+        </is>
+      </c>
+      <c r="B177" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D177" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" s="9">
+        <f>SUMIF(Escandallos!$C$4:$C$331,A177,Escandallos!$G$4:$G$331)</f>
+        <v/>
+      </c>
+      <c r="F177" s="9">
+        <f>C177+D177-E177</f>
+        <v/>
+      </c>
+      <c r="G177" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="9">
+        <f>G177-F177</f>
+        <v/>
+      </c>
+      <c r="I177" s="14">
+        <f>IFERROR(H177/F177,0)</f>
+        <v/>
+      </c>
+      <c r="J177" s="15">
+        <f>IF(ABS(I177)&gt;$B$2,"Revisar","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C172" s="17">
-        <f>SUM(C5:C170)</f>
-        <v/>
-      </c>
-      <c r="D172" s="17">
-        <f>SUM(D5:D170)</f>
-        <v/>
-      </c>
-      <c r="E172" s="17">
-        <f>SUM(E5:E170)</f>
-        <v/>
-      </c>
-      <c r="F172" s="17">
-        <f>SUM(F5:F170)</f>
-        <v/>
-      </c>
-      <c r="G172" s="17">
-        <f>SUM(G5:G170)</f>
-        <v/>
-      </c>
-      <c r="H172" s="17">
-        <f>SUM(H5:H170)</f>
-        <v/>
-      </c>
-      <c r="J172" s="18">
-        <f>COUNTIF(J5:J170,"Revisar")&amp;" ingrediente(s) a revisar"</f>
+      <c r="B179" s="6" t="n"/>
+      <c r="C179" s="13">
+        <f>SUM(C5:C177)</f>
+        <v/>
+      </c>
+      <c r="D179" s="13">
+        <f>SUM(D5:D177)</f>
+        <v/>
+      </c>
+      <c r="E179" s="9">
+        <f>SUM(E5:E177)</f>
+        <v/>
+      </c>
+      <c r="F179" s="9">
+        <f>SUM(F5:F177)</f>
+        <v/>
+      </c>
+      <c r="G179" s="13">
+        <f>SUM(G5:G177)</f>
+        <v/>
+      </c>
+      <c r="H179" s="9">
+        <f>SUM(H5:H177)</f>
+        <v/>
+      </c>
+      <c r="I179" s="14" t="n"/>
+      <c r="J179" s="15">
+        <f>COUNTIF(J5:J177,"Revisar")&amp;" ingrediente(s) a revisar"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>CONSUMIBLES — seguimiento directo por compras y recuento (limpieza, papel, envases; no vinculado a ventas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="8" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B182" s="8" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="inlineStr">
+        <is>
+          <t>Stock mes anterior</t>
+        </is>
+      </c>
+      <c r="D182" s="8" t="inlineStr">
+        <is>
+          <t>Compras del mes</t>
+        </is>
+      </c>
+      <c r="E182" s="8" t="inlineStr">
+        <is>
+          <t>Stock final (recuento real)</t>
+        </is>
+      </c>
+      <c r="F182" s="8" t="inlineStr">
+        <is>
+          <t>Consumo real del mes</t>
+        </is>
+      </c>
+      <c r="G182" s="8" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>Servilletas de papel</t>
+        </is>
+      </c>
+      <c r="B183" s="6" t="inlineStr">
+        <is>
+          <t>PAQ</t>
+        </is>
+      </c>
+      <c r="C183" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D183" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" s="9">
+        <f>C183+D183-E183</f>
+        <v/>
+      </c>
+      <c r="G183" s="13">
+        <f>IF(F183&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>EJEMPLO — sustituir por el listado real de consumibles de Lady Madrid (confirmar con cocina/sala)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>Papel de horno</t>
+        </is>
+      </c>
+      <c r="B184" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E184" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" s="9">
+        <f>C184+D184-E184</f>
+        <v/>
+      </c>
+      <c r="G184" s="13">
+        <f>IF(F184&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="inlineStr">
+        <is>
+          <t>Film transparente</t>
+        </is>
+      </c>
+      <c r="B185" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" s="9">
+        <f>C185+D185-E185</f>
+        <v/>
+      </c>
+      <c r="G185" s="13">
+        <f>IF(F185&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>Bolsas de basura</t>
+        </is>
+      </c>
+      <c r="B186" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C186" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E186" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" s="9">
+        <f>C186+D186-E186</f>
+        <v/>
+      </c>
+      <c r="G186" s="13">
+        <f>IF(F186&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
+        <is>
+          <t>Guantes de nitrilo</t>
+        </is>
+      </c>
+      <c r="B187" s="6" t="inlineStr">
+        <is>
+          <t>CAJA</t>
+        </is>
+      </c>
+      <c r="C187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E187" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" s="9">
+        <f>C187+D187-E187</f>
+        <v/>
+      </c>
+      <c r="G187" s="13">
+        <f>IF(F187&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="6" t="inlineStr">
+        <is>
+          <t>Detergente lavavajillas</t>
+        </is>
+      </c>
+      <c r="B188" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E188" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" s="9">
+        <f>C188+D188-E188</f>
+        <v/>
+      </c>
+      <c r="G188" s="13">
+        <f>IF(F188&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="inlineStr">
+        <is>
+          <t>Envases take away</t>
+        </is>
+      </c>
+      <c r="B189" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C189" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" s="9">
+        <f>C189+D189-E189</f>
+        <v/>
+      </c>
+      <c r="G189" s="13">
+        <f>IF(F189&lt;0,"Revisar (recuento negativo)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>Vasos y tapas para llevar</t>
+        </is>
+      </c>
+      <c r="B190" s="6" t="inlineStr">
+        <is>
+          <t>UD</t>
+        </is>
+      </c>
+      <c r="C190" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E190" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" s="9">
+        <f>C190+D190-E190</f>
+        <v/>
+      </c>
+      <c r="G190" s="13">
+        <f>IF(F190&lt;0,"Revisar (recuento negativo)","")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A181:G181"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>